<commit_message>
Deploy Smart Card Cross-Referencing Engine: Linked 911 Folio ECA26072301237 with WhatsApp Card and Deduplicated
</commit_message>
<xml_diff>
--- a/historico_c5/tarjetas_informativas/CONCENTRADO_MASTER_TARJETAS_INFORMATIVAS.xlsx
+++ b/historico_c5/tarjetas_informativas/CONCENTRADO_MASTER_TARJETAS_INFORMATIVAS.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,51 @@
           <t>id_tarjeta</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>victima</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>edad</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>casquillos</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>policia_unidad</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ubicacion</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>imagen_path</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>folio_911_vinculado</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>incidente_911</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>coincidencia_estatus</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -487,6 +532,153 @@
       <c r="G2" t="inlineStr">
         <is>
           <t>TI-20260728_133304</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ECATEPEC</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ECATEPEC (PERSONA MUERTA POR IMPACTOS DE BALA)
+A las 10:55 horas, el Policía GUTIERREZ RAMIREZ JUAN CARLOS unidad ME334A, informó que, en calle Colorines esquina calle Encino, colonia Tierra Blanca, hizo contacto con el Primer Respondiente Policía Municipal FERMÍN GUZMÁN FERNANDO unidad sector 3-21, indicando de una persona muerta por impactos de bala, quien respondía al nombre de RICARDO HERNÁNDEZ MAYA REYNOSA de 33 años, localizándose en el lugar 5 casquillos percutidos de calibre 9mm; arribo personal de Protección Civil unidad PC-2021, al mando del Paramédico JUAN CARLOS GALVÁN, quien certifica que ya no cuentan con signos vitales.</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-07-28 13:36:18</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>RICARDO HERNÁNDEZ MAYA REYNOSA</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>33</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>5 casquillos calibre 9m</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>GUTIERREZ RAMIREZ JUAN CARLOS (ME334A)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>calle Colorines esquina calle Encino, colonia Tierra Blanca</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>whatsapp_ecatepec_colorines.png</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>ECA26072301237</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>ACCIDENTE DE TRANSITO SIN PERSONAS LESIONADAS</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>VINCULADA 911 C5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>23:55</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TECÁMAC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TECÁMAC (PERSONA MUERTA POR IMPACTO DE BALA)
+A las 23:55 horas, el Policía MALDONADO SUÁREZ JUAN TRINIDAD, unidad ME937A5, informó que a las 06:15 horas, en calle Jardines de La Viña esquina 2da. Cerrada de Jardines de La Viña, fraccionamiento Héroes Tecámac, hizo contacto con la Primer Respondiente Policía Municipal NORMA HERNÁNDEZ CASTRO unidad C-072, quien toma conocimiento de una persona muerta quien en vida respondía al nombre de LUIS EDUARDO RUIZ ROJAS de 35 años, el cual se encuentra a bordo de un vehículo marca Chevrolet, tipo Chevy Monza, color blanco, placas PUB383E, con bandera de taxi, localizando 7 casquillos percutidos calibre 9mm, arribo la Unidad Médica PC-70, al mando de la Paramédico ROCIÓ ZARATE RANGEL, indicando que ya no cuenta con signos vitales, debido a los impactos que presenta en la cara, indica la Primer Respondiente que se trató de un intento de asalto y al oponer resistencia le disparan.</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-07-28 13:36:26</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>LUIS EDUARDO RUIZ ROJAS</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>35</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>7 casquillos 9mm</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Municipal NORMA HERNÁNDEZ CASTRO (C-072)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>No especificada</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>whatsapp_tecamac_chevy.png</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>SIN REGISTRO PREVIO 911</t>
         </is>
       </c>
     </row>

</xml_diff>